<commit_message>
Describe every ritual and detail the Booqme handover
All seventeen rituals now carry an "O rituále" description, up from four.
The Booqme workbook gains full service descriptions ready to paste, a
fourteen-step admin guide naming each field, voucher types including a
discount code, and a category overview.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ty41EDx4pQ4VhbjBYSdEXf
</commit_message>
<xml_diff>
--- a/docs/booqme-programy.xlsx
+++ b/docs/booqme-programy.xlsx
@@ -10,6 +10,7 @@
     <sheet name="Programy" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Poukážky" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Postup v Booqme" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Prehľad ponuky" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -33,16 +34,19 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
+      <sz val="10"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -52,6 +56,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001B2A24"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FDF6E6"/>
       </patternFill>
     </fill>
   </fills>
@@ -81,10 +90,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -92,13 +104,19 @@
     <xf numFmtId="164" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -464,563 +482,899 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="44" customWidth="1" min="5" max="5"/>
-    <col width="70" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="44" customWidth="1" min="6" max="6"/>
+    <col width="78" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
+    <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Kategória (Booqme: Kategória služby)</t>
+          <t>Č.</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Kategória služby</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Názov služby</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Dĺžka trvania (min)</t>
-        </is>
-      </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>Trvanie (min)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>Cena (€)</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Krátky popis (pod názov)</t>
-        </is>
-      </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Popis služby (čo rituál obsahuje)</t>
+          <t>Krátky popis</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Odporúčané (zvýrazniť)</t>
+          <t>Popis služby (do poľa Popis v Booqme)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Odporúčané</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>Head Spa rituály</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>Klasický Head Spa</t>
         </is>
       </c>
-      <c r="C2" s="2" t="n">
+      <c r="D2" s="2" t="n">
         <v>40</v>
       </c>
-      <c r="D2" s="3" t="n">
+      <c r="E2" s="4" t="n">
         <v>50</v>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="F2" s="3" t="inlineStr">
         <is>
           <t>Krátky a príjemný Head Spa zážitok pre chvíľu oddychu a profesionálnu starostlivosť o vlasy a pokožku hlavy.</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Rituál obsahuje: Uvítací nápoj · Krátka konzultácia · Jemný peeling pokožky hlavy · Čistenie pokožky hlavy · Relaxačná masáž hlavy · Jemný vodný Head Spa rituál · Umytie vlasov · Hydratačná starostlivosť · Teplý uterákový rituál · Záverečné vysušenie vlasov</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr"/>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>Prvých štyridsať minút, počas ktorých zistíte, prečo sa o Head Spa hovorí. Krátky, ale úplný rituál: peeling, hĺbkové čistenie pokožky hlavy, relaxačná masáž a vodný rituál v teplej vode.
+Ideálny, ak si chcete Head Spa vyskúšať prvýkrát, alebo si doprajete oddych medzi dvoma pracovnými dňami. Odchádzate s čistou pokožkou hlavy, upravenými vlasmi a hlavou o niečo ľahšou.
+Rituál obsahuje:
+• Uvítací nápoj
+• Krátka konzultácia
+• Jemný peeling pokožky hlavy
+• Čistenie pokožky hlavy
+• Relaxačná masáž hlavy
+• Jemný vodný Head Spa rituál
+• Umytie vlasov
+• Hydratačná starostlivosť
+• Teplý uterákový rituál
+• Záverečné vysušenie vlasov</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>Head Spa rituály</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>Relaxačný Head Spa</t>
         </is>
       </c>
-      <c r="C3" s="2" t="n">
+      <c r="D3" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="D3" s="3" t="n">
+      <c r="E3" s="4" t="n">
         <v>70</v>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>60 minút pokojného rituálu s dôrazom na fyzické aj psychické uvoľnenie.</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>Doprajte si 60 minút, počas ktorých sa svet na chvíľu zastaví. Relaxačný Head Spa rituál je vytvorený v pokojnej atmosfére, s dôrazom na ticho, jemný dotyk, vôňu, teplo a vodu. Postupné uvoľnenie pokožky hlavy, tváre a dekoltu prináša príjemný pocit ľahkosti a oddychu.
-Rituál obsahuje: Uvítací nápoj · Aromaterapeutický úvod · Peeling a hĺbkové čistenie pokožky hlavy · Relaxačná masáž hlavy · Rituál so sérom na pokožku hlavy · Masáž tváre · Relaxačná masáž dekoltu · Teplý uterákový rituál · Luxusný vodný Head Spa rituál · Výživná vlasová maska · Chladivý očný rituál · Záverečné opláchnutie a profesionálne vysušenie vlasov</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr"/>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Doprajte si 60 minút, počas ktorých sa svet na chvíľu zastaví. Relaxačný Head Spa rituál je vytvorený v pokojnej atmosfére, s dôrazom na ticho, jemný dotyk, vôňu, teplo a vodu.
+Postupné uvoľnenie pokožky hlavy, tváre a dekoltu prináša príjemný pocit ľahkosti a oddychu.
+Rituál obsahuje:
+• Uvítací nápoj
+• Aromaterapeutický úvod
+• Peeling a hĺbkové čistenie pokožky hlavy
+• Relaxačná masáž hlavy
+• Rituál so sérom na pokožku hlavy
+• Masáž tváre
+• Relaxačná masáž dekoltu
+• Teplý uterákový rituál
+• Luxusný vodný Head Spa rituál
+• Výživná vlasová maska
+• Chladivý očný rituál
+• Záverečné opláchnutie a profesionálne vysušenie vlasov</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>Head Spa rituály</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>Head Spa harmónia</t>
         </is>
       </c>
-      <c r="C4" s="2" t="n">
+      <c r="D4" s="2" t="n">
         <v>75</v>
       </c>
-      <c r="D4" s="3" t="n">
+      <c r="E4" s="4" t="n">
         <v>85</v>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>Komplexný relaxačný rituál, v ktorom sa spája voda, teplo, vôňa, jemný dotyk a ticho.</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>Rituál obsahuje: Uvítací nápoj · Aromaterapeutický úvod · Jemný peeling a osvieženie pokožky hlavy · Intenzívna relaxačná masáž hlavy · Masáž tváre a spánkov · Teplý bylinný obklad · Luxusný vodný Head Spa rituál · Hĺbkový hydratačný vlasový zábal · Relaxačný zvukový rituál · Uvoľňujúci záverečný rituál pokoja · Záverečné opláchnutie a profesionálne vysušenie vlasov</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr"/>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Sedemdesiatpäť minút bez ponáhľania. Rituál postupne prechádza od pokožky hlavy cez spánky a tvár až k tichu.
+Teplý bylinný obklad, hĺbkový hydratačný zábal a relaxačný zvukový rituál držia telo aj myseľ v jednom pokojnom tempe.
+Vhodné vtedy, keď máte za sebou náročné obdobie a potrebujete viac než len rýchly oddych.
+Rituál obsahuje:
+• Uvítací nápoj
+• Aromaterapeutický úvod
+• Jemný peeling a osvieženie pokožky hlavy
+• Intenzívna relaxačná masáž hlavy
+• Masáž tváre a spánkov
+• Teplý bylinný obklad
+• Luxusný vodný Head Spa rituál
+• Hĺbkový hydratačný vlasový zábal
+• Relaxačný zvukový rituál
+• Uvoľňujúci záverečný rituál pokoja
+• Záverečné opláchnutie a profesionálne vysušenie vlasov</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>Head Spa rituály</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>Hĺbkový rituál pre pokožku hlavy</t>
         </is>
       </c>
-      <c r="C5" s="2" t="n">
+      <c r="D5" s="2" t="n">
         <v>90</v>
       </c>
-      <c r="D5" s="3" t="n">
+      <c r="E5" s="4" t="n">
         <v>95</v>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>Prémiová starostlivosť pre pokožku, ktorá pôsobí zaťažene, nadmerne sa mastí, má sklony k lupinám alebo potrebuje intenzívnejšiu očistu.</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>Rituál obsahuje: Uvítací nápoj · Úvodná konzultácia a rozhovor o stave pokožky hlavy · Trichologické pozorovanie pokožky hlavy kamerou · Jemný predčistiaci rituál · Hĺbkový detox pokožky hlavy · Peeling podľa aktuálneho stavu pokožky · Relaxačná a stimulačná masáž pokožky hlavy · Teplý uterákový rituál · Špeciálna čistiaca starostlivosť pre pokožku hlavy · Vodný Head Spa rituál · Ošetrenie pokožky vhodným sérom · Výživná starostlivosť pre vlasy · Relaxačný záverečný rituál v tichu · Profesionálne vysušenie vlasov</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr"/>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Rituál pre pokožku, ktorá pôsobí zaťažene, rýchlo sa mastí, svrbí alebo má sklony k lupinám.
+Začíname rozhovorom a pozorovaním pokožky hlavy trichologickou kamerou, aby sme videli jej skutočný stav. Podľa toho vyberáme peeling aj následnú starostlivosť.
+Nasleduje hĺbkový detox, stimulačná masáž, vodný Head Spa rituál a sérum zvolené presne pre vašu pokožku. Deväťdesiat minút, po ktorých pokožka hlavy konečne dýcha.
+Rituál obsahuje:
+• Uvítací nápoj
+• Úvodná konzultácia a rozhovor o stave pokožky hlavy
+• Trichologické pozorovanie pokožky hlavy kamerou
+• Jemný predčistiaci rituál
+• Hĺbkový detox pokožky hlavy
+• Peeling podľa aktuálneho stavu pokožky
+• Relaxačná a stimulačná masáž pokožky hlavy
+• Teplý uterákový rituál
+• Špeciálna čistiaca starostlivosť pre pokožku hlavy
+• Vodný Head Spa rituál
+• Ošetrenie pokožky vhodným sérom
+• Výživná starostlivosť pre vlasy
+• Relaxačný záverečný rituál v tichu
+• Profesionálne vysušenie vlasov</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>Head Spa rituály</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>Kozmetický Head Spa rituál</t>
         </is>
       </c>
-      <c r="C6" s="2" t="n">
+      <c r="D6" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="D6" s="3" t="n">
+      <c r="E6" s="4" t="n">
         <v>75</v>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Kompletný beauty &amp; relax zážitok pre pokožku hlavy, tvár aj vlasy.</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>Rituál obsahuje: Uvítací nápoj · Aromaterapeutický úvod · Jemné čistenie pokožky hlavy · Relaxačná masáž hlavy a spánkov · Luxusný vodný Head Spa rituál · Čistiaca a hydratačná maska na tvár · Liftingová masáž tváre · Relaxačná masáž dekoltu · Teplý uterákový rituál · Výživná maska pre vlasy · Chladivý očný rituál · Intenzívny záverečný pleťový rituál · Záverečné opláchnutie a profesionálne vysušenie vlasov</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr"/>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>Spojenie Head Spa a kozmetiky v jednej hodine. Staráme sa o pokožku hlavy, tvár aj vlasy naraz.
+Čistiaca a hydratačná maska, liftingová masáž tváre a relaxačná masáž dekoltu dopĺňajú klasický vodný rituál.
+Voľba pre tých, ktorí chcú z jednej návštevy odísť oddýchnutí aj rozžiarení.
+Rituál obsahuje:
+• Uvítací nápoj
+• Aromaterapeutický úvod
+• Jemné čistenie pokožky hlavy
+• Relaxačná masáž hlavy a spánkov
+• Luxusný vodný Head Spa rituál
+• Čistiaca a hydratačná maska na tvár
+• Liftingová masáž tváre
+• Relaxačná masáž dekoltu
+• Teplý uterákový rituál
+• Výživná maska pre vlasy
+• Chladivý očný rituál
+• Intenzívny záverečný pleťový rituál
+• Záverečné opláchnutie a profesionálne vysušenie vlasov</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Head Spa rituály</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>Ovocný a osviežujúci Head Spa rituál</t>
         </is>
       </c>
-      <c r="C7" s="2" t="n">
+      <c r="D7" s="2" t="n">
         <v>75</v>
       </c>
-      <c r="D7" s="3" t="n">
+      <c r="E7" s="4" t="n">
         <v>89</v>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>Hravý, svieži a zároveň luxusný rituál spájajúci ovocie, vodu, vôňu, teplo a dotyk.</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>Rituál obsahuje: Uvítací nápoj s čerstvým ovocím · Svieži aromatický úvod · Rituál s čerstvým sezónnym ovocím · Jemné čistenie pokožky hlavy · Relaxačná masáž hlavy a spánkov · Luxusný vodný Head Spa rituál · Chladivý uhorkový očný rituál · Svieži pleťový obklad · Relaxačná masáž tváre · Teplý uterákový rituál · Čerstvý ovocný vlasový zábal · Hydratačná vlasová starostlivosť · Jemný aromatický záverečný rituál · Profesionálne vysušenie vlasov</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr"/>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Rituál, ktorý je cítiť a dá sa aj ochutnať. Pracujeme s čerstvým sezónnym ovocím, chladivou uhorkou a sviežimi vôňami.
+Teplo a chlad sa striedajú, ovocný vlasový zábal a svieži pleťový obklad zanechajú pokožku osviežanú a vlasy vyživené.
+Obľúbená voľba na jar a v lete, aj ako darček pre niekoho, kto má rád niečo iné než klasiku.
+Rituál obsahuje:
+• Uvítací nápoj s čerstvým ovocím
+• Svieži aromatický úvod
+• Rituál s čerstvým sezónnym ovocím
+• Jemné čistenie pokožky hlavy
+• Relaxačná masáž hlavy a spánkov
+• Luxusný vodný Head Spa rituál
+• Chladivý uhorkový očný rituál
+• Svieži pleťový obklad
+• Relaxačná masáž tváre
+• Teplý uterákový rituál
+• Čerstvý ovocný vlasový zábal
+• Hydratačná vlasová starostlivosť
+• Jemný aromatický záverečný rituál
+• Profesionálne vysušenie vlasov</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>Head Spa rituály</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>Prémiový Head Spa rituál</t>
         </is>
       </c>
-      <c r="C8" s="2" t="n">
+      <c r="D8" s="2" t="n">
         <v>120</v>
       </c>
-      <c r="D8" s="3" t="n">
+      <c r="E8" s="4" t="n">
         <v>149</v>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="F8" s="3" t="inlineStr">
         <is>
           <t>Dve hodiny premysleného zážitku od pokožky hlavy cez tvár a vlasy až k chodidlám.</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>Rituál obsahuje: Uvítací nápoj · Privítací aromaterapeutický rituál s výberom vône · Jemný peeling a hĺbkové očistenie pokožky hlavy · Luxusný vodný Head Spa rituál · Intenzívny relaxačný rituál pokožky hlavy · Rituál pre spánky a tvár · Luxusná pleťová maska · Chladivý očný rituál · Teplý aromatický uterákový rituál · Hĺbkový vlasový zábal podľa typu vlasov · Výživné sérum pre pokožku hlavy · Reflexný rituál pre chodidlá · Hrejivý zábal chodidiel · Jemný tlakový rituál chodidiel · Relaxačný zvukový rituál · Tichý aromaterapeutický odpočinok · Luxusné záverečné ošetrenie vlasov · Profesionálne vysušenie a finálna úprava</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>Dve hodiny, počas ktorých neriešite nič. Najkompletnejší rituál, aký v HEAD SPA 30 ponúkame.
+Začíname výberom vône a hĺbkovým očistením pokožky hlavy, pokračujeme luxusným vodným rituálom, starostlivosťou o tvár a oči a vlasovým zábalom podľa typu vlasov.
+Záver patrí chodidlám: reflexný rituál, hrejivý zábal a jemné tlakové techniky. Všetko uzatvára zvukový rituál a tichý aromaterapeutický odpočinok.
+Ak si chcete dopriať Head Spa v jeho najúplnejšej podobe, toto je ono.
+Rituál obsahuje:
+• Uvítací nápoj
+• Privítací aromaterapeutický rituál s výberom vône
+• Jemný peeling a hĺbkové očistenie pokožky hlavy
+• Luxusný vodný Head Spa rituál
+• Intenzívny relaxačný rituál pokožky hlavy
+• Rituál pre spánky a tvár
+• Luxusná pleťová maska
+• Chladivý očný rituál
+• Teplý aromatický uterákový rituál
+• Hĺbkový vlasový zábal podľa typu vlasov
+• Výživné sérum pre pokožku hlavy
+• Reflexný rituál pre chodidlá
+• Hrejivý zábal chodidiel
+• Jemný tlakový rituál chodidiel
+• Relaxačný zvukový rituál
+• Tichý aromaterapeutický odpočinok
+• Luxusné záverečné ošetrenie vlasov
+• Profesionálne vysušenie a finálna úprava</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>áno</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>Pánske rituály</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>Pánsky Head Spa</t>
         </is>
       </c>
-      <c r="C9" s="2" t="n">
+      <c r="D9" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="D9" s="3" t="n">
+      <c r="E9" s="4" t="n">
         <v>55</v>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="F9" s="3" t="inlineStr">
         <is>
           <t>45 minút pokoja, sviežosti a starostlivosti vytvorenej špeciálne pre mužov.</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>Rituál obsahuje: Uvítací nápoj · Úvodný relaxačný rituál · Jemný peeling pokožky hlavy · Hĺbkové čistenie pokožky hlavy · Relaxačný rituál hlavy a spánkov · Luxusný vodný Head Spa rituál · Teplý uterákový rituál · Osviežujúce ošetrenie pokožky hlavy · Výživná starostlivosť pre vlasy · Záverečné opláchnutie a profesionálne vysušenie vlasov</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr"/>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>Štyridsaťpäť minút vytvorených pre mužov. Bez zbytočností, ale s plnou starostlivosťou.
+Peeling, hĺbkové čistenie pokožky hlavy, relaxačný rituál hlavy a spánkov, luxusný vodný rituál a teplý uterák.
+Ideálne po práci alebo pred dôležitým dňom. Pokožka hlavy je čistá, vlasy svieže a hlava vypnutá.
+Rituál obsahuje:
+• Uvítací nápoj
+• Úvodný relaxačný rituál
+• Jemný peeling pokožky hlavy
+• Hĺbkové čistenie pokožky hlavy
+• Relaxačný rituál hlavy a spánkov
+• Luxusný vodný Head Spa rituál
+• Teplý uterákový rituál
+• Osviežujúce ošetrenie pokožky hlavy
+• Výživná starostlivosť pre vlasy
+• Záverečné opláchnutie a profesionálne vysušenie vlasov</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>Pánske rituály</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>Pánsky harmonický rituál</t>
         </is>
       </c>
-      <c r="C10" s="2" t="n">
+      <c r="D10" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="D10" s="3" t="n">
+      <c r="E10" s="4" t="n">
         <v>75</v>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="F10" s="3" t="inlineStr">
         <is>
           <t>Drevité a svieže tóny, teplý uterák, voda a jemný dotyk vytvárajú atmosféru moderného pánskeho relax.</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>Rituál obsahuje: Uvítací nápoj · Výber charakteristickej pánskej vône: drevo, céder, bergamot · Osviežujúci peeling pokožky hlavy · Hĺbkové čistenie pokožky hlavy · Relaxačný rituál hlavy a spánkov · Luxusný vodný Head Spa rituál · Hrejivý aromatický uterákový rituál · Chladivý očný rituál · Relaxačný rituál pre tvár · Výživná vlasová starostlivosť · Ošetrenie pokožky hlavy pánskym sérom · Záverečný relaxačný moment v tichu · Profesionálne vysušenie vlasov</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr"/>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>Hodina v drevitých a sviežich tónoch. Na začiatku si vyberiete vôňu: drevo, céder alebo bergamot.
+Teplý aromatický uterák, chladivý očný rituál a relaxačný rituál pre tvár dopĺňajú luxusný vodný Head Spa rituál.
+Rituál končí niekoľkými minútami v úplnom tichu. Práve tie si muži pochvaľujú najviac.
+Rituál obsahuje:
+• Uvítací nápoj
+• Výber charakteristickej pánskej vône: drevo, céder, bergamot
+• Osviežujúci peeling pokožky hlavy
+• Hĺbkové čistenie pokožky hlavy
+• Relaxačný rituál hlavy a spánkov
+• Luxusný vodný Head Spa rituál
+• Hrejivý aromatický uterákový rituál
+• Chladivý očný rituál
+• Relaxačný rituál pre tvár
+• Výživná vlasová starostlivosť
+• Ošetrenie pokožky hlavy pánskym sérom
+• Záverečný relaxačný moment v tichu
+• Profesionálne vysušenie vlasov</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>Pánske rituály</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>Pánsky hĺbkový rituál pre pokožku hlavy</t>
         </is>
       </c>
-      <c r="C11" s="2" t="n">
+      <c r="D11" s="2" t="n">
         <v>90</v>
       </c>
-      <c r="D11" s="3" t="n">
+      <c r="E11" s="4" t="n">
         <v>99</v>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="F11" s="3" t="inlineStr">
         <is>
           <t>90 minút dôkladnej starostlivosti pre mužov, ktorí chcú pokožke hlavy vrátiť pocit čistoty, sviežosti a komfortu.</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="G11" s="3" t="inlineStr">
         <is>
           <t>90 minút dôkladnej starostlivosti pre mužov, ktorí chcú svoju pokožku hlavy dostať späť do pocitu čistoty, sviežosti a komfortu.
-Rituál obsahuje: Uvítací nápoj · Úvodná konzultácia · Trichologické pozorovanie pokožky hlavy kamerou · Analýza aktuálneho stavu pokožky · Predčistiaci rituál · Hĺbkový peeling pokožky hlavy · Detoxikačné čistenie · Relaxačný rituál hlavy a spánkov · Luxusný vodný Head Spa rituál · Teplý aromatický uterákový rituál · Cielená starostlivosť pri nadmernom mastení, lupinách a nánosoch stylingových produktov · Ošetrenie pokožky vhodným sérom · Výživná starostlivosť pre vlasy · Chladivý očný rituál · Záverečný relax v tichu · Profesionálne vysušenie vlasov</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr"/>
+Začíname konzultáciou a pozorovaním pokožky hlavy trichologickou kamerou. Až podľa toho, čo na nej vidíme, volíme peeling, detox aj sérum.
+Rituál cielene rieši nadmerné mastenie, lupiny a nánosy stylingových produktov. Medzi jednotlivými krokmi je priestor na teplý uterák, chladivý očný rituál a záverečný oddych v tichu.
+Rituál obsahuje:
+• Uvítací nápoj
+• Úvodná konzultácia
+• Trichologické pozorovanie pokožky hlavy kamerou
+• Analýza aktuálneho stavu pokožky
+• Predčistiaci rituál
+• Hĺbkový peeling pokožky hlavy
+• Detoxikačné čistenie
+• Relaxačný rituál hlavy a spánkov
+• Luxusný vodný Head Spa rituál
+• Teplý aromatický uterákový rituál
+• Cielená starostlivosť pri nadmernom mastení, lupinách a nánosoch stylingových produktov
+• Ošetrenie pokožky vhodným sérom
+• Výživná starostlivosť pre vlasy
+• Chladivý očný rituál
+• Záverečný relax v tichu
+• Profesionálne vysušenie vlasov</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>Pánske rituály</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="C12" s="3" t="inlineStr">
         <is>
           <t>Prémiový pánsky rituál</t>
         </is>
       </c>
-      <c r="C12" s="2" t="n">
+      <c r="D12" s="2" t="n">
         <v>120</v>
       </c>
-      <c r="D12" s="3" t="n">
+      <c r="E12" s="4" t="n">
         <v>149</v>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="F12" s="3" t="inlineStr">
         <is>
           <t>Dve hodiny bez telefónov a zhonu. Jeden plynulý pánsky relaxačný zážitok od pokožky hlavy až po chodidlá.</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>Dve hodiny, počas ktorých nemusíte nič riešiť. Rituál je vytvorený pre muža, ktorý si chce dopriať najvyššiu úroveň komfortu, oddychu a starostlivosti. Začíname pri pokožke hlavy a postupne prechádzame cez vlasy, tvár a oči až k chodidlám. Teplé uteráky, voda, drevité vône, vlasové zábaly, pleťová maska a starostlivosť o chodidlá vytvárajú jeden plynulý zážitok. Počas rituálu je priestor na ticho, pokoj a úplné vypnutie. Žiadne telefóny, žiadny zhon, iba dve hodiny venované vám. Odpočívate. My sa postaráme o zvyšok. Keď obyčajný relax nestačí a chcete zažiť Head Spa v jeho najluxusnejšej podobe.
-Rituál obsahuje: Uvítací nápoj · Výber charakteristickej pánskej vône: céder, santalové drevo, bergamot · Úvodný rituál na spomalenie a uvoľnenie · Jemný peeling pokožky hlavy · Luxusný vodný Head Spa rituál · Intenzívny relaxačný rituál hlavy a spánkov · Teplý aromatický uterákový rituál · Luxusná hydratačná maska na tvár · Chladivý očný rituál · Hĺbkový vlasový zábal · Výživné sérum pre pokožku hlavy · Relaxačný reflexný rituál pre chodidlá · Hrejivý zábal chodidiel · Regeneračná maska na chodidlá · Jemný tlakový rituál chodidiel · Aromatický oddych v tichu · Relaxačný zvukový rituál · Záverečná vlasová starostlivosť · Profesionálne vysušenie a finálna úprava</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>Dve hodiny, počas ktorých nemusíte nič riešiť.
+Rituál je vytvorený pre muža, ktorý si chce dopriať najvyššiu úroveň komfortu, oddychu a starostlivosti.
+Začíname pri pokožke hlavy a postupne prechádzame cez vlasy, tvár a oči až k chodidlám. Teplé uteráky, voda, drevité vône, vlasové zábaly, pleťová maska a starostlivosť o chodidlá vytvárajú jeden plynulý zážitok.
+Počas rituálu je priestor na ticho, pokoj a úplné vypnutie. Žiadne telefóny, žiadny zhon, iba dve hodiny venované vám.
+Odpočívate. My sa postaráme o zvyšok. Keď obyčajný relax nestačí a chcete zažiť Head Spa v jeho najluxusnejšej podobe.
+Rituál obsahuje:
+• Uvítací nápoj
+• Výber charakteristickej pánskej vône: céder, santalové drevo, bergamot
+• Úvodný rituál na spomalenie a uvoľnenie
+• Jemný peeling pokožky hlavy
+• Luxusný vodný Head Spa rituál
+• Intenzívny relaxačný rituál hlavy a spánkov
+• Teplý aromatický uterákový rituál
+• Luxusná hydratačná maska na tvár
+• Chladivý očný rituál
+• Hĺbkový vlasový zábal
+• Výživné sérum pre pokožku hlavy
+• Relaxačný reflexný rituál pre chodidlá
+• Hrejivý zábal chodidiel
+• Regeneračná maska na chodidlá
+• Jemný tlakový rituál chodidiel
+• Aromatický oddych v tichu
+• Relaxačný zvukový rituál
+• Záverečná vlasová starostlivosť
+• Profesionálne vysušenie a finálna úprava</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>áno</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>Detské rituály</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr">
         <is>
           <t>Detský ovocný Head Spa</t>
         </is>
       </c>
-      <c r="C13" s="2" t="n">
+      <c r="D13" s="2" t="n">
         <v>50</v>
       </c>
-      <c r="D13" s="3" t="n">
+      <c r="E13" s="4" t="n">
         <v>55</v>
       </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="F13" s="3" t="inlineStr">
         <is>
           <t>Hravý a nežný rituál vytvorený špeciálne pre deti: voňavo, jemne a s úsmevom.</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>Rituál obsahuje: Detský welcome drink · Ovocný aromatický úvod · Jemné čistenie pokožky hlavy · Ovocný vlasový zábal · Jemný relaxačný rituál hlavy · Jemný vodný Head Spa rituál · Jemná masáž hlavy · Teplý uteráčikový rituál · Hydratačná starostlivosť o vlasy · Malý relaxačný oddych · Záverečné umytie a vysušenie vlasov</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr"/>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>Rituál vytvorený tak, aby sa v ňom deti cítili bezpečne a zároveň ich to bavilo.
+Ovocné vône, detský uvítací nápoj, jemné čistenie pokožky hlavy, ovocný vlasový zábal a teplý uteráčik. Všetko jemne, pomaly a s úsmevom.
+Vhodné pre deti, ktoré vydržia pokojne poležať. Rodič môže zostať v miestnosti po celý čas.
+Rituál obsahuje:
+• Detský welcome drink
+• Ovocný aromatický úvod
+• Jemné čistenie pokožky hlavy
+• Ovocný vlasový zábal
+• Jemný relaxačný rituál hlavy
+• Jemný vodný Head Spa rituál
+• Jemná masáž hlavy
+• Teplý uteráčikový rituál
+• Hydratačná starostlivosť o vlasy
+• Malý relaxačný oddych
+• Záverečné umytie a vysušenie vlasov</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>Rituály pre dvoch</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="C14" s="3" t="inlineStr">
         <is>
           <t>Spoločný Head Spa rituál</t>
         </is>
       </c>
-      <c r="C14" s="2" t="n">
+      <c r="D14" s="2" t="n">
         <v>652</v>
       </c>
-      <c r="D14" s="3" t="n">
+      <c r="E14" s="4" t="n">
         <v>129</v>
       </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="F14" s="3" t="inlineStr">
         <is>
           <t>Spoločný oddych pre partnerov, manželov, mamu a dcéru, sestry, kamarátky či mamu a syna.</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>Rituál obsahuje: Uvítací nápoj pre oboch · Aromaterapeutický úvod · Výber vône podľa nálady · Jemný peeling pokožky hlavy · Hĺbkové čistenie pokožky hlavy · Relaxačný rituál hlavy a spánkov · Luxusný vodný Head Spa rituál · Teplý aromatický uterákový rituál · Hydratačná vlasová maska · Jemný rituál pre tvár · Chladivý očný rituál · Krátky relaxačný zvukový rituál · Výživné záverečné ošetrenie vlasov · Profesionálne vysušenie vlasov</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr"/>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>Rituál pre dvoch, vedľa seba. Partneri, manželia, mama s dcérou, sestry, kamarátky alebo mama so synom.
+Každý si na začiatku vyberie vôňu podľa nálady, potom už len ležíte. Rozprávať sa nemusíte.
+Uvedená cena platí za obe osoby.
+Rituál obsahuje:
+• Uvítací nápoj pre oboch
+• Aromaterapeutický úvod
+• Výber vône podľa nálady
+• Jemný peeling pokožky hlavy
+• Hĺbkové čistenie pokožky hlavy
+• Relaxačný rituál hlavy a spánkov
+• Luxusný vodný Head Spa rituál
+• Teplý aromatický uterákový rituál
+• Hydratačná vlasová maska
+• Jemný rituál pre tvár
+• Chladivý očný rituál
+• Krátky relaxačný zvukový rituál
+• Výživné záverečné ošetrenie vlasov
+• Profesionálne vysušenie vlasov</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>Rituály pre dvoch</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="C15" s="3" t="inlineStr">
         <is>
           <t>Spoločný rituál pod hviezdami</t>
         </is>
       </c>
-      <c r="C15" s="2" t="n">
+      <c r="D15" s="2" t="n">
         <v>752</v>
       </c>
-      <c r="D15" s="3" t="n">
+      <c r="E15" s="4" t="n">
         <v>149</v>
       </c>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="F15" s="3" t="inlineStr">
         <is>
           <t>Rituál pre dvoch v tlmenom svetle s hviezdnou oblohou, vôňou, teplom, vodou a pokojnými zvukmi.</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>Rituál obsahuje: Uvítací nápoj pre oboch · Výber vône pre spoločný aromaterapeutický úvod · Jemný peeling pokožky hlavy · Hĺbkové čistenie pokožky hlavy · Relaxačný rituál hlavy a spánkov · Luxusný vodný Head Spa rituál · Teplý aromatický uterákový rituál · Hydratačná vlasová maska s teplým turbanom · Jemný relaxačný rituál pre tvár · Chladivý očný rituál · Rituál pod hviezdnou oblohou · Pokojný zvukový sprievod a tlmené svetlo · Záverečné výživné ošetrenie vlasov · Profesionálne vysušenie vlasov</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>Sedemdesiatpäť minút v tlmenom svetle pod hviezdnou oblohou.
+K spoločnému Head Spa rituálu pridávame hydratačnú masku s teplým turbanom, hviezdnu atmosféru a pokojný zvukový sprievod.
+Najčastejšie sa daruje k výročiu či Valentínovi, alebo len tak, keď chcete niekoho prekvapiť. Uvedená cena platí za obe osoby.
+Rituál obsahuje:
+• Uvítací nápoj pre oboch
+• Výber vône pre spoločný aromaterapeutický úvod
+• Jemný peeling pokožky hlavy
+• Hĺbkové čistenie pokožky hlavy
+• Relaxačný rituál hlavy a spánkov
+• Luxusný vodný Head Spa rituál
+• Teplý aromatický uterákový rituál
+• Hydratačná vlasová maska s teplým turbanom
+• Jemný relaxačný rituál pre tvár
+• Chladivý očný rituál
+• Rituál pod hviezdnou oblohou
+• Pokojný zvukový sprievod a tlmené svetlo
+• Záverečné výživné ošetrenie vlasov
+• Profesionálne vysušenie vlasov</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
         <is>
           <t>áno</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>Rituály pre chodidlá</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="C16" s="3" t="inlineStr">
         <is>
           <t>Klasický rituál pre chodidlá</t>
         </is>
       </c>
-      <c r="C16" s="2" t="n">
+      <c r="D16" s="2" t="n">
         <v>40</v>
       </c>
-      <c r="D16" s="3" t="n">
+      <c r="E16" s="4" t="n">
         <v>45</v>
       </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="F16" s="3" t="inlineStr">
         <is>
           <t>40 minút úplného vypnutia s dôrazom na pocit uvoľnenia, ľahkosti a sviežosti chodidiel.</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="G16" s="3" t="inlineStr">
         <is>
           <t>Doprajte svojim nohám viac než len oddych. Doprajte si chvíľu úplného vypnutia.
-Rituál obsahuje: Uvítací nápoj · Voňavý aromaterapeutický úvod · Teplý kúpeľ chodidiel · Jemné penové očistenie · Peeling chodidiel · Osviežujúca maska na chodidlá · Hydratačná maska na päty · Teplý uterákový zábal · Reflexný tlakový rituál chodidiel · Jemné stimulačné techniky na chodidlách · Výživné sérum a intenzívna hydratácia · Záverečný relaxačný rituál v tichu</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr"/>
+Štyridsať minút, počas ktorých sa chodidlá dostanú z teplého kúpeľa cez peeling a masku až k reflexnému tlakovému rituálu.
+Teplý uterákový zábal, výživné sérum a intenzívna hydratácia zanechajú chodidlá hladké a ľahké. Rituál končí niekoľkými minútami v tichu.
+Rituál obsahuje:
+• Uvítací nápoj
+• Voňavý aromaterapeutický úvod
+• Teplý kúpeľ chodidiel
+• Jemné penové očistenie
+• Peeling chodidiel
+• Osviežujúca maska na chodidlá
+• Hydratačná maska na päty
+• Teplý uterákový zábal
+• Reflexný tlakový rituál chodidiel
+• Jemné stimulačné techniky na chodidlách
+• Výživné sérum a intenzívna hydratácia
+• Záverečný relaxačný rituál v tichu</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+      <c r="A17" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>Rituály pre chodidlá</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="C17" s="3" t="inlineStr">
         <is>
           <t>Ovocný a bylinkový rituál pre chodidlá</t>
         </is>
       </c>
-      <c r="C17" s="2" t="n">
+      <c r="D17" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="D17" s="3" t="n">
+      <c r="E17" s="4" t="n">
         <v>65</v>
       </c>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="F17" s="3" t="inlineStr">
         <is>
           <t>Svieži, voňavý a prírodne ladený rituál, v ktorom sa teplo postupne strieda s osviežením.</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>Rituál obsahuje: Uvítací nápoj s čerstvým ovocím · Voňavý aromaterapeutický úvod · Teplý bylinný kúpeľ chodidiel s čerstvými citrusmi · Jemné penové očistenie · Ovocný peeling chodidiel · Čerstvý ovocný a bylinný obklad · Chladivý osviežujúci rituál · Hydratačná maska na chodidlá a päty · Teplý uterákový zábal · Reflexný tlakový rituál chodidiel · Jemné stimulačné techniky pre pocit uvoľnenia · Výživné ovocné maslo/krémové ošetrenie · Aromaterapeutický oddych v tichu · Záverečný relaxačný rituál</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr"/>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>Hodina pre chodidlá, v ktorej sa teplo strieda s osviežením.
+Teplý bylinný kúpeľ s čerstvými citrusmi, ovocný peeling, bylinný obklad, hydratačná maska a reflexný tlakový rituál.
+Odchádzate s pocitom, že ste celý deň stáli na tráve, nie na asfalte.
+Rituál obsahuje:
+• Uvítací nápoj s čerstvým ovocím
+• Voňavý aromaterapeutický úvod
+• Teplý bylinný kúpeľ chodidiel s čerstvými citrusmi
+• Jemné penové očistenie
+• Ovocný peeling chodidiel
+• Čerstvý ovocný a bylinný obklad
+• Chladivý osviežujúci rituál
+• Hydratačná maska na chodidlá a päty
+• Teplý uterákový zábal
+• Reflexný tlakový rituál chodidiel
+• Jemné stimulačné techniky pre pocit uvoľnenia
+• Výživné ovocné maslo/krémové ošetrenie
+• Aromaterapeutický oddych v tichu
+• Záverečný relaxačný rituál</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+      <c r="A18" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
         <is>
           <t>Rituály pre chodidlá</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="C18" s="3" t="inlineStr">
         <is>
           <t>Zlatý rituál 24K</t>
         </is>
       </c>
-      <c r="C18" s="2" t="n">
+      <c r="D18" s="2" t="n">
         <v>90</v>
       </c>
-      <c r="D18" s="3" t="n">
+      <c r="E18" s="4" t="n">
         <v>119</v>
       </c>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="F18" s="3" t="inlineStr">
         <is>
           <t>90 minút absolútneho rozmaznávania. 24-karátové zlato, teplo, vôňa, dotyk a ticho.</t>
         </is>
       </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>Rituál obsahuje: Uvítací nápoj · Zlatý aromaterapeutický úvod · Teplý kúpeľ chodidiel s minerálnym a aromatickým rituálom · Jemné penové očistenie · Luxusný peeling chodidiel · 24K zlatý peelingový rituál · Teplý uterákový zábal · Zlatá hydratačná maska na chodidlá · 24K zlatý zábal na päty a chodidlá · Reflexný tlakový rituál chodidiel · Jemné stimulačné techniky pre pocit uvoľnenia · Výživné sérum obohatené o kozmetické zlato · Hrejivý zábal chodidiel · Chladivý záverečný rituál · Aromaterapeutický odpočinok v úplnom tichu · Luxusné záverečné ošetrenie chodidiel</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="inlineStr">
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>Deväťdesiat minút absolútneho rozmaznávania s kozmetickým 24-karátovým zlatom.
+Zlatý peelingový rituál, zlatá hydratačná maska a zábal na päty a chodidlá, doplnené teplom, vôňou a reflexnou masážou.
+Náš najluxusnejší rituál pre chodidlá. Obľúbený ako darček vtedy, keď chcete darovať niečo naozaj výnimočné.
+Rituál obsahuje:
+• Uvítací nápoj
+• Zlatý aromaterapeutický úvod
+• Teplý kúpeľ chodidiel s minerálnym a aromatickým rituálom
+• Jemné penové očistenie
+• Luxusný peeling chodidiel
+• 24K zlatý peelingový rituál
+• Teplý uterákový zábal
+• Zlatá hydratačná maska na chodidlá
+• 24K zlatý zábal na päty a chodidlá
+• Reflexný tlakový rituál chodidiel
+• Jemné stimulačné techniky pre pocit uvoľnenia
+• Výživné sérum obohatené o kozmetické zlato
+• Hrejivý zábal chodidiel
+• Chladivý záverečný rituál
+• Aromaterapeutický odpočinok v úplnom tichu
+• Luxusné záverečné ošetrenie chodidiel</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
         <is>
           <t>áno</t>
         </is>
@@ -1037,157 +1391,238 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="70" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="62" customWidth="1" min="5" max="5"/>
+    <col width="62" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>Názov typu poukážky</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="5" t="inlineStr">
         <is>
           <t>Druh v Booqme</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Hodnota (€)</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Platnosť (mesiace)</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>Hodnota</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>Platnosť</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
         <is>
           <t>Popis pre zákazníka</t>
         </is>
       </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>Poznámka</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>Darčekový poukaz 50 €</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>Predplatený kredit</t>
         </is>
       </c>
-      <c r="C2" s="2" t="n">
-        <v>50</v>
-      </c>
-      <c r="D2" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Kredit 50 € na ľubovoľný Head Spa rituál v HEAD SPA 30, Mostná 30, Nitra. Kód zadáte pri online rezervácii.</t>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>50 €</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>12 mesiacov</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Kredit 50 € na ľubovoľný rituál v HEAD SPA 30, Mostná 30, Nitra. Šesťmiestny kód zadáte pri online rezervácii.</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Zvyšok kreditu zostáva na ďalšiu návštevu.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Darčekový poukaz 70 €</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>Predplatený kredit</t>
         </is>
       </c>
-      <c r="C3" s="2" t="n">
-        <v>70</v>
-      </c>
-      <c r="D3" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Kredit 70 € na ľubovoľný Head Spa rituál v HEAD SPA 30, Mostná 30, Nitra. Kód zadáte pri online rezervácii.</t>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>70 €</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>12 mesiacov</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Kredit 70 € na ľubovoľný rituál v HEAD SPA 30, Mostná 30, Nitra. Šesťmiestny kód zadáte pri online rezervácii.</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Zvyšok kreditu zostáva na ďalšiu návštevu.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Darčekový poukaz 100 €</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>Predplatený kredit</t>
         </is>
       </c>
-      <c r="C4" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="D4" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>Kredit 100 € na ľubovoľný Head Spa rituál v HEAD SPA 30, Mostná 30, Nitra. Kód zadáte pri online rezervácii.</t>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>100 €</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>12 mesiacov</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Kredit 100 € na ľubovoľný rituál v HEAD SPA 30, Mostná 30, Nitra. Šesťmiestny kód zadáte pri online rezervácii.</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Zvyšok kreditu zostáva na ďalšiu návštevu.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Darčekový poukaz 149 €</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>Predplatený kredit</t>
         </is>
       </c>
-      <c r="C5" s="2" t="n">
-        <v>149</v>
-      </c>
-      <c r="D5" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>Kredit 149 € na ľubovoľný Head Spa rituál v HEAD SPA 30, Mostná 30, Nitra. Kód zadáte pri online rezervácii.</t>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>149 €</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>12 mesiacov</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Kredit 149 € na ľubovoľný rituál v HEAD SPA 30, Mostná 30, Nitra. Šesťmiestny kód zadáte pri online rezervácii.</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Zvyšok kreditu zostáva na ďalšiu návštevu.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Darčekový poukaz na rituál</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Voľný počet vstupov (1)</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Poukaz na konkrétny rituál</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Voľný počet vstupov (1 vstup)</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>podľa rituálu</t>
         </is>
       </c>
-      <c r="D6" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>Jeden konkrétny rituál podľa výberu (napr. Prémiový Head Spa rituál). Vytvorte samostatný typ pre každý rituál, ktorý chcete darovať.</t>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>12 mesiacov</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Jeden konkrétny rituál podľa výberu, napríklad Prémiový Head Spa rituál.</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Vytvorte samostatný typ pre každý rituál, ktorý chcete ponúkať ako darček. Odporúčame štyri najžiadanejšie: Prémiový Head Spa rituál, Prémiový pánsky rituál, Spoločný rituál pod hviezdami, Zlatý rituál 24K.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Zľava 10 % na prvú návštevu</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Zľavový kód</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>10 %</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>podľa kampane</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Desaťpercentná zľava z celej rezervácie.</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Nepovinné. Vhodné na akcie a spolupráce.</t>
         </is>
       </c>
     </row>
@@ -1202,116 +1637,438 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="110" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="105" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
-        <is>
-          <t>Časť</t>
-        </is>
-      </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>Krok</t>
         </is>
       </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Kde v Booqme</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>Čo presne spraviť</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="inlineStr">
-        <is>
-          <t>Programy (služby)</t>
-        </is>
-      </c>
-      <c r="B2" s="6" t="inlineStr">
-        <is>
-          <t>1. Prihláste sa na https://booqme.app/sk/prihlasenie účtom pre Barbershop 30 (Head Spa).</t>
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>Prihlásenie</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Otvorte booqme.app/sk/prihlasenie a prihláste sa účtom salónu (redstylenitra@gmail.com). Ak máte v účte dve prevádzky, vyberte tú s pracovníkom Salón 30 - Head SPA Nitra, jej rezervačná stránka je booqme.app/sk/rezervacia/barbershop-30.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr"/>
-      <c r="B3" s="6" t="inlineStr">
-        <is>
-          <t>2. V menu otvorte Služby a najprv vytvorte 5 kategórií z hárku Programy (stĺpec A).</t>
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>Služby, kategórie</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Najprv vytvorte päť kategórií presne v tomto poradí: Head Spa rituály, Pánske rituály, Detské rituály, Rituály pre dvoch, Rituály pre chodidlá. Poradie kategórií určuje, v akom poradí ich uvidí zákazník.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr"/>
-      <c r="B4" s="6" t="inlineStr">
-        <is>
-          <t>3. Pre každý riadok hárku Programy kliknite Pridať službu: názov, kategória, dĺžka trvania v minútach, cena. Krátky popis a Popis služby skopírujte zo stĺpcov E a F.</t>
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Služby, pridať službu</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Pre každý z 17 riadkov hárku Programy kliknite Pridať službu a vyplňte: Názov (stĺpec C), Kategória (stĺpec B), Dĺžka trvania (stĺpec D, v minútach), Cena (stĺpec E), Popis (stĺpec G, skopírujte celý text aj so zoznamom krokov).</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr"/>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>4. Pri službe priraďte pracovníka „Salón 30 - Head SPA Nitra“ a podľa potreby zapnite platbu kartou vopred (celá suma alebo záloha).</t>
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Služby, pracovník</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Pri každej službe zaškrtnite pracovníka Salón 30 - Head SPA Nitra, inak sa služba zákazníkom nezobrazí v kalendári.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr"/>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>5. Testovaciu službu „trvala“ (60 min, 45 €) zmažte alebo skryte, aby sa nezobrazovala zákazníkom.</t>
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Služby, rituály pre dvoch</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Pri službách Spoločný Head Spa rituál a Spoločný rituál pod hviezdami je cena za dve osoby. Ak Booqme ponúka pole Počet osôb, nastavte 2. Inak doplňte do popisu vetu, že cena platí za obe osoby (v texte už je).</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>Poukážky online</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>6. V menu otvorte Darčekové poukážky a vytvorte typy z hárku Poukážky. Odporúčaný druh je Predplatený kredit (zákazník ho môže minúť aj na viac návštev).</t>
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Služby, platby</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Rozhodnite sa, či chcete pri rezervácii zálohu. Odporúčame zálohu pri rituáloch nad 100 €, teda pri Prémiovom Head Spa rituáli, Prémiovom pánskom rituáli, Spoločnom rituáli pod hviezdami a Zlatom rituáli 24K. Zálohu nastavíte pri službe ako pevnú sumu alebo percento.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr"/>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>7. Po vytvorení typov sa v rezervačnom formulári automaticky objaví možnosť Kúpiť darčekovú poukážku. Platba kartou beží cez Stripe Connect (v Nastaveniach prepojte alebo založte Stripe účet). Poplatok je od 1,99 % z platby, minimálna platba 3 €.</t>
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Služby, upratanie</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Zmažte alebo skryte testovaciu službu trvala (60 min, 45 €), aby ju zákazníci nevideli.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr"/>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>8. Zákazník dostane poukaz s 6-miestnym kódom e-mailom. Obdarovaný ho zadá pri rezervácii, prípadne ho zadáte ručne pri telefonickej rezervácii.</t>
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Nastavenia, Stripe</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Aby sa dali poukážky a zálohy platiť kartou, prepojte Stripe účet cez Stripe Connect. Peniaze chodia priamo na váš účet, Booqme ich nedrží. Poplatok je od 1,99 % z platby (0,49 % Booqme plus sadzba Stripe), minimálna platba je 3 €.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="inlineStr">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Darčekové poukážky</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Vytvorte typy poukážok z hárku Poukážky. Pre každý zadajte názov, druh, hodnotu, platnosť a popis. Odporúčaný druh je Predplatený kredit, zákazník ho môže minúť aj na viac návštev.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Darčekové poukážky, kontrola</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Po uložení otvorte booqme.app/sk/rezervacia/barbershop-30 v anonymnom okne. V rezervačnom formulári musí pribudnúť možnosť kúpiť darčekovú poukážku. Ak tam nie je, typy poukážok nie sú aktívne.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Poukážky v salóne</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Poukážky sa dajú vygenerovať a vytlačiť aj vopred a predávať priamo na prevádzke. Takáto poukážka nie je aktívna, kým ju v systéme neoznačíte ako predanú.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Uplatnenie poukazu</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Zákazník zadá šesťmiestny kód pri online rezervácii. Pri telefonickej rezervácii kód zadáte vy ručne, dá sa doplniť aj dodatočne.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
         <is>
           <t>Web</t>
         </is>
       </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>9. Web HEAD SPA 30 už odkazuje na https://booqme.app/sk/rezervacia/barbershop-30 zo všetkých tlačidiel Rezervovať aj z tlačidla Kúpiť poukaz online. Nič ďalšie netreba meniť.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="5" t="inlineStr"/>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t>10. Ak sa zmení názov alebo adresa rezervačnej stránky v Booqme, treba nahradiť odkaz na webe (README, sekcia Rezervácie).</t>
-        </is>
-      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Na webe už nie je čo meniť. Všetky tlačidlá Rezervovať aj tlačidlo Kúpiť poukaz online vedú na booqme.app/sk/rezervacia/barbershop-30. Web je živý na d8f5s88zjy-art.github.io/head-spa-30.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Kontrola na záver</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>V anonymnom okne prejdite celú rezerváciu ako zákazník: vyberte rituál, termín, vyplňte údaje a zastavte sa pred platbou. Skontrolujte, či sedí názov, dĺžka, cena a popis.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Kategória</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Počet rituálov</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>Najnižšia cena</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>Najvyššia cena</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>Rozsah trvania</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t>Head Spa rituály</t>
+        </is>
+      </c>
+      <c r="B2" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="C2" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="D2" s="9" t="n">
+        <v>149</v>
+      </c>
+      <c r="E2" s="8" t="inlineStr">
+        <is>
+          <t>40 až 120 min</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>Pánske rituály</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="C3" s="9" t="n">
+        <v>55</v>
+      </c>
+      <c r="D3" s="9" t="n">
+        <v>149</v>
+      </c>
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>45 až 120 min</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>Detské rituály</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" s="9" t="n">
+        <v>55</v>
+      </c>
+      <c r="D4" s="9" t="n">
+        <v>55</v>
+      </c>
+      <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>50 až 50 min</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>Rituály pre dvoch</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="C5" s="9" t="n">
+        <v>129</v>
+      </c>
+      <c r="D5" s="9" t="n">
+        <v>149</v>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>652 až 752 min</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>Rituály pre chodidlá</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="C6" s="9" t="n">
+        <v>45</v>
+      </c>
+      <c r="D6" s="9" t="n">
+        <v>119</v>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>40 až 90 min</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>Spolu</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="n">
+        <v>17</v>
+      </c>
+      <c r="C7" s="11" t="n">
+        <v>45</v>
+      </c>
+      <c r="D7" s="11" t="n">
+        <v>149</v>
+      </c>
+      <c r="E7" s="10" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>